<commit_message>
La nomenclature publique descend à la source : aucun livrable ne parle plus en sigles
scenarios.py porte la traduction unique (public_id, public_col) : S1/S2/S3
restent les identifiants internes du pipeline, mais tout fichier écrit dans
livrables/ dit base / recommande / reference-interne, colonnes comprises
(vmax_recommande_kmh_plafond_courbure, bande_geometrie_base, t_base_cap160_min).
Les cartes, le KMZ, les LISEZMOI et les popups suivent ; les lecteurs (12, 19,
24, 28, 32) lisent les nouveaux noms ; le visualiseur affiche zéro sigle, fil
et 24 tables balayés au navigateur, quatre vérifications au vert. Et
« accel_laterale_m_s2 » s'affiche désormais comme l'unité qu'il est (m/s²),
pas comme un scénario.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/livrables/blocs_urbains.xlsx
+++ b/livrables/blocs_urbains.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>HYPOTHÈSE : fenêtre km, traversée au plafond S1 ∧ bande</t>
+          <t>HYPOTHÈSE : fenêtre km, traversée au plafond du scénario de base ∧ bande</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>HYPOTHÈSE : fenêtre km, traversée au plafond S1 ∧ bande</t>
+          <t>HYPOTHÈSE : fenêtre km, traversée au plafond du scénario de base ∧ bande</t>
         </is>
       </c>
     </row>

</xml_diff>